<commit_message>
copy: polish delegated wording for PR #86
</commit_message>
<xml_diff>
--- a/docs/reviews/2026-10-22-r03-radar-copy-workbook.xlsx
+++ b/docs/reviews/2026-10-22-r03-radar-copy-workbook.xlsx
@@ -495,7 +495,7 @@
       </c>
       <c r="B1" s="2" t="n"/>
     </row>
-    <row r="2">
+    <row r="2" ht="24" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
           <t>Trạng thái</t>
@@ -503,7 +503,7 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>BẢN NHÁP. Chưa nối vào code, chưa vào kho nền đã duyệt (fallback-approval). Không câu nào hiển thị cho người dùng cho tới khi owner duyệt và một PR riêng nối vào renderer.</t>
+          <t xml:space="preserve">Đã có quyết định theo uỷ quyền ngày 26/10/2026; Codex rà câu chữ, Claude review bản sửa. Chưa nối vào renderer hay kho fallback. Giọng thứ tư là deep_dive; 140 câu roast không dùng.</t>
         </is>
       </c>
     </row>
@@ -1653,7 +1653,7 @@
         </is>
       </c>
     </row>
-    <row r="11">
+    <row r="11" ht="60" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
           <t>R03-moon-square-sun-partner-gentle_specific</t>
@@ -1745,7 +1745,7 @@
       </c>
       <c r="T11" s="6" t="inlineStr">
         <is>
-          <t>Uỷ quyền 26/10: viết lại → Có những tối bạn cần được vỗ về đúng lúc người yêu hào hứng kể việc vừa làm xong; nói ra bạn cần gì sẽ nhẹ hơn. (Đoán ý người kia: “người yêu muốn được khen” gán nhu cầu bên trong như sự thật; thay bằng hành vi quan sát được (hào hứng kể). “thứ tự mong muốn” hơi cứng.). Codex chuốt trước khi wiring</t>
+          <t xml:space="preserve">Uỷ quyền 26/10: viết lại → Có những tối bạn cần được vỗ về lúc người yêu hào hứng kể việc vừa xong; nói rõ bạn cần gì để cả hai cùng biết. | Codex chuốt 26/10; Claude review trước khi wiring.</t>
         </is>
       </c>
     </row>
@@ -2037,7 +2037,7 @@
         </is>
       </c>
     </row>
-    <row r="15">
+    <row r="15" ht="60" customHeight="1">
       <c r="A15" s="4" t="inlineStr">
         <is>
           <t>R03-moon-square-sun-someone-gentle_specific</t>
@@ -2129,11 +2129,11 @@
       </c>
       <c r="T15" s="6" t="inlineStr">
         <is>
-          <t>Uỷ quyền 26/10: viết lại → Nếu bạn đang cần yên mà người này lại hào hứng kể nhiều chuyện, quá tải đến nhanh; nhận ra sớm giúp bạn chọn lúc dừng. (Bản cũ hơi phán xét (“kể chuyện mình không ngừng”)). Codex chuốt trước khi wiring</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
+          <t xml:space="preserve">Uỷ quyền 26/10: viết lại → Nếu bạn đang cần yên mà người này kể liền nhiều chuyện, bạn có thể thấy quá tải; nói rõ khi mình cần dừng. | Codex chuốt 26/10; Claude review trước khi wiring.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="60" customHeight="1">
       <c r="A16" s="4" t="inlineStr">
         <is>
           <t>R03-moon-square-sun-someone-playful_grounded</t>
@@ -2225,7 +2225,7 @@
       </c>
       <c r="T16" s="6" t="inlineStr">
         <is>
-          <t>Uỷ quyền 26/10: viết lại → Người này hào hứng kể liền mấy chuyện, bạn thì đang muốn yên: chào tạm biệt lịch sự cũng là một kỹ năng. (Bản cũ chế giễu người kia (“phát trực tiếp chuyện đời họ”)). Codex chuốt trước khi wiring</t>
+          <t xml:space="preserve">Uỷ quyền 26/10: viết lại → Người này kể liền mấy chuyện, bạn thì muốn yên một chút: hôm nay xin phép tan ca nghe chuyện sớm. | Codex chuốt 26/10; Claude review trước khi wiring.</t>
         </is>
       </c>
     </row>
@@ -2517,7 +2517,7 @@
         </is>
       </c>
     </row>
-    <row r="20">
+    <row r="20" ht="60" customHeight="1">
       <c r="A20" s="4" t="inlineStr">
         <is>
           <t>R03-true_node-square-sun-crush-playful_grounded</t>
@@ -2609,7 +2609,7 @@
       </c>
       <c r="T20" s="6" t="inlineStr">
         <is>
-          <t>Uỷ quyền 26/10: viết lại → Bạn đang tập sống chậm, crush lại sống như phim hành động: kịch bản mới của bạn bị thử lửa hơi sớm. (Sai nghĩa: “bị thử vai” (thử vai = casting) không ra ý “bị thử thách”.). Codex chuốt trước khi wiring</t>
+          <t xml:space="preserve">Uỷ quyền 26/10: viết lại → Bạn đang tập sống chậm mà đã gật đầu theo crush đi khắp nơi: lịch mới thử được ba ngày, khoan nhận thêm kèo. | Codex chuốt 26/10; Claude review trước khi wiring.</t>
         </is>
       </c>
     </row>
@@ -2805,7 +2805,7 @@
         </is>
       </c>
     </row>
-    <row r="23">
+    <row r="23" ht="60" customHeight="1">
       <c r="A23" s="4" t="inlineStr">
         <is>
           <t>R03-true_node-square-sun-friend-gentle_specific</t>
@@ -2897,7 +2897,7 @@
       </c>
       <c r="T23" s="6" t="inlineStr">
         <is>
-          <t>Uỷ quyền 26/10: viết lại → Có thể cá tính rõ ràng của bạn ấy làm bạn lưỡng lự với hướng mình đang đi; kể bạn ấy nghe và hỏi bạn ấy hỗ trợ được gì. (“cái tôi rõ ràng” trong tiếng Việt thường mang nghĩa chê (ego), nghe như nhận xét xấu về bạn ấy; mục ma sát nên là “dễ cấn”, không phải “xấu”.). Codex chuốt trước khi wiring</t>
+          <t xml:space="preserve">Uỷ quyền 26/10: viết lại → Nếu lời rủ của bạn ấy làm bạn lưỡng lự với hướng đang đi, kể rõ điều bạn đang tập và hỏi bạn ấy có thể hỗ trợ gì. | Codex chuốt 26/10; Claude review trước khi wiring.</t>
         </is>
       </c>
     </row>
@@ -3093,7 +3093,7 @@
         </is>
       </c>
     </row>
-    <row r="26">
+    <row r="26" ht="60" customHeight="1">
       <c r="A26" s="4" t="inlineStr">
         <is>
           <t>R03-true_node-square-sun-partner-straight_warm</t>
@@ -3185,11 +3185,11 @@
       </c>
       <c r="T26" s="6" t="inlineStr">
         <is>
-          <t>Uỷ quyền 26/10: viết lại → Khi bạn muốn đổi hướng sống, nếp sống người yêu đã quen có thể tạo ma sát; nói rõ thay đổi đó quan trọng với bạn ra sao. (Câu lủng củng: “cách người yêu đã quen là chính mình” không tự nhiên.). Codex chuốt trước khi wiring</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
+          <t xml:space="preserve">Uỷ quyền 26/10: viết lại → Khi bạn muốn đổi hướng sống, nếp quen của người yêu có thể khiến hai người khó thống nhất; nói rõ thay đổi nào quan trọng với bạn. | Codex chuốt 26/10; Claude review trước khi wiring.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="60" customHeight="1">
       <c r="A27" s="4" t="inlineStr">
         <is>
           <t>R03-true_node-square-sun-partner-gentle_specific</t>
@@ -3281,7 +3281,7 @@
       </c>
       <c r="T27" s="6" t="inlineStr">
         <is>
-          <t>Uỷ quyền 26/10: viết lại → Có thể khi bạn kể về hướng mới, người yêu đáp lại dè dặt hơn bạn nghĩ; hỏi xem thay đổi đó chạm vào điều gì của hai người. (Đoán nội tâm: “chạm vào hình ảnh họ đang giữ” là suy đoán về người yêu, trừu tượng, không quan sát được; khung “hình ảnh … đang giữ” lặp lại.). Codex chuốt trước khi wiring</t>
+          <t xml:space="preserve">Uỷ quyền 26/10: viết lại → Có thể khi bạn kể hướng mới, người yêu hỏi lại nhiều hơn bạn nghĩ; hỏi xem thay đổi nào hai người cần bàn thêm. | Codex chuốt 26/10; Claude review trước khi wiring.</t>
         </is>
       </c>
     </row>
@@ -4053,7 +4053,7 @@
         </is>
       </c>
     </row>
-    <row r="36">
+    <row r="36" ht="60" customHeight="1">
       <c r="A36" s="4" t="inlineStr">
         <is>
           <t>R03-jupiter-trine-pluto-crush-playful_grounded</t>
@@ -4145,7 +4145,7 @@
       </c>
       <c r="T36" s="6" t="inlineStr">
         <is>
-          <t>Uỷ quyền 26/10: viết lại → Crush kể về nỗi sợ lớn nhất, bạn nghe hết rồi mới hỏi có muốn cùng nghĩ cách không: lạc quan đúng lúc, khá ổn. (Bản cũ khen đáp nỗi sợ bằng kế hoạch, trái các câu “nghe trước”). Codex chuốt trước khi wiring</t>
+          <t xml:space="preserve">Uỷ quyền 26/10: viết lại → Crush kể nỗi sợ, bạn nghe hết rồi mới hỏi có muốn cùng nghĩ cách không: đội cứu hộ hôm nay nhớ xin phép trước. | Codex chuốt 26/10; Claude review trước khi wiring.</t>
         </is>
       </c>
     </row>
@@ -5781,7 +5781,7 @@
         </is>
       </c>
     </row>
-    <row r="54">
+    <row r="54" ht="60" customHeight="1">
       <c r="A54" s="4" t="inlineStr">
         <is>
           <t>R03-jupiter-trine-sun-friend-straight_warm</t>
@@ -5873,7 +5873,7 @@
       </c>
       <c r="T54" s="6" t="inlineStr">
         <is>
-          <t>Uỷ quyền 26/10: viết lại → Khi bạn ấy đứng trước quyết định lớn, bạn thường là người lên tiếng tin bạn ấy đầu tiên; nói điều đó thật rõ, đừng để bạn ấy phải đoán. (Đoán nội tâm: “tin vào bạn ấy nhiều hơn chính bạn ấy” khẳng định bạn ấy thiếu tự tin như sự thật.). Codex chuốt trước khi wiring</t>
+          <t xml:space="preserve">Uỷ quyền 26/10: viết lại → Khi bạn ấy đứng trước quyết định lớn, một lời động viên cụ thể của bạn có thể giúp ích; hỏi bạn ấy muốn nghe hay cần góp ý. | Codex chuốt 26/10; Claude review trước khi wiring.</t>
         </is>
       </c>
     </row>
@@ -5973,7 +5973,7 @@
         </is>
       </c>
     </row>
-    <row r="56">
+    <row r="56" ht="60" customHeight="1">
       <c r="A56" s="4" t="inlineStr">
         <is>
           <t>R03-jupiter-trine-sun-friend-playful_grounded</t>
@@ -6065,7 +6065,7 @@
       </c>
       <c r="T56" s="6" t="inlineStr">
         <is>
-          <t>Uỷ quyền 26/10: viết lại → Bạn ấy nói muốn đi hát, bạn đã đặt luôn sân khấu: quản lý tài năng tự phong. (“bẩm sinh” gợi tính cách định sẵn từ khi sinh, gần định mệnh trong bối cảnh lá số; “tự phong” giữ chất đùa.). Codex chuốt trước khi wiring</t>
+          <t xml:space="preserve">Uỷ quyền 26/10: viết lại → Bạn ấy vừa nhắc chuyện đi hát, bạn đã xung phong đặt phòng: quản lý tự phong nhớ hỏi ca sĩ trước. | Codex chuốt 26/10; Claude review trước khi wiring.</t>
         </is>
       </c>
     </row>
@@ -7029,7 +7029,7 @@
         </is>
       </c>
     </row>
-    <row r="67">
+    <row r="67" ht="60" customHeight="1">
       <c r="A67" s="4" t="inlineStr">
         <is>
           <t>R03-mercury-square-sun-crush-gentle_specific</t>
@@ -7121,7 +7121,7 @@
       </c>
       <c r="T67" s="6" t="inlineStr">
         <is>
-          <t>Uỷ quyền 26/10: viết lại → Một câu góp ý nhỏ khi nhắn tin có thể rơi đúng vào điều crush vừa hào hứng khoe; chậm lại một nhịp khi chọn chữ. (Đoán ý người kia: “điều crush đang muốn được công nhận” gán nhu cầu bên trong; thay bằng hành vi thấy được (vừa khoe).). Codex chuốt trước khi wiring</t>
+          <t xml:space="preserve">Uỷ quyền 26/10: viết lại → Một câu góp ý khi nhắn tin có thể đến ngay lúc crush vừa khoe thành quả; ghi nhận việc ấy trước khi hỏi thêm. | Codex chuốt 26/10; Claude review trước khi wiring.</t>
         </is>
       </c>
     </row>
@@ -7797,7 +7797,7 @@
         </is>
       </c>
     </row>
-    <row r="75">
+    <row r="75" ht="60" customHeight="1">
       <c r="A75" s="4" t="inlineStr">
         <is>
           <t>R03-mercury-square-sun-partner-gentle_specific</t>
@@ -7889,7 +7889,7 @@
       </c>
       <c r="T75" s="6" t="inlineStr">
         <is>
-          <t>Uỷ quyền 26/10: viết lại → Những lời nhận xét bạn thấy rất bình thường có thể rơi đúng lúc người yêu đang khoe việc vừa làm được; để ý phản ứng ngay sau câu đó. (Đoán ý người kia: “chỗ người yêu đang muốn được tự hào” gán nhu cầu bên trong, câu cũng hơi tối nghĩa.). Codex chuốt trước khi wiring</t>
+          <t xml:space="preserve">Uỷ quyền 26/10: viết lại → Lời nhận xét bạn thấy bình thường có thể đến lúc người yêu vừa khoe việc làm được; để ý phản ứng rồi hỏi lại nếu chưa rõ. | Codex chuốt 26/10; Claude review trước khi wiring.</t>
         </is>
       </c>
     </row>
@@ -8181,7 +8181,7 @@
         </is>
       </c>
     </row>
-    <row r="79">
+    <row r="79" ht="60" customHeight="1">
       <c r="A79" s="4" t="inlineStr">
         <is>
           <t>R03-mercury-square-sun-someone-gentle_specific</t>
@@ -8273,7 +8273,7 @@
       </c>
       <c r="T79" s="6" t="inlineStr">
         <is>
-          <t>Uỷ quyền 26/10: viết lại → Có thể câu hỏi thẳng của bạn đến đúng lúc người này đang kể điều họ làm tốt; một câu ghi nhận trước giúp câu hỏi được nghe đúng ý. (Đoán nội tâm: “hình ảnh người này đang giữ” không quan sát được; khung “hình ảnh … đang giữ” lặp với true_node-square-sun-partner.). Codex chuốt trước khi wiring</t>
+          <t xml:space="preserve">Uỷ quyền 26/10: viết lại → Nếu câu hỏi thẳng của bạn đến lúc người này kể việc làm tốt, ghi nhận phần cụ thể trước rồi mới hỏi thêm. | Codex chuốt 26/10; Claude review trước khi wiring.</t>
         </is>
       </c>
     </row>
@@ -9717,7 +9717,7 @@
         </is>
       </c>
     </row>
-    <row r="95">
+    <row r="95" ht="60" customHeight="1">
       <c r="A95" s="4" t="inlineStr">
         <is>
           <t>R03-mercury-trine-true_node-someone-gentle_specific</t>
@@ -9809,7 +9809,7 @@
       </c>
       <c r="T95" s="6" t="inlineStr">
         <is>
-          <t>Uỷ quyền 26/10: viết lại → Nếu bạn để ý, có thể sau vài câu bạn nói người này hỏi thêm về một hướng mới; cứ chia sẻ, không cần biết trước kết quả. (Không quan sát được: “khiến người này nghĩ về một hướng mới” nói về suy nghĩ người kia; đổi sang hành vi (hỏi thêm).). Codex chuốt trước khi wiring</t>
+          <t xml:space="preserve">Uỷ quyền 26/10: viết lại → Nếu sau vài câu bạn nói, người này hỏi thêm về một hướng mới, cứ chia sẻ điều mình biết và để họ tự chọn. | Codex chuốt 26/10; Claude review trước khi wiring.</t>
         </is>
       </c>
     </row>
@@ -12885,7 +12885,7 @@
         </is>
       </c>
     </row>
-    <row r="128">
+    <row r="128" ht="60" customHeight="1">
       <c r="A128" s="4" t="inlineStr">
         <is>
           <t>R03-sun-trine-venus-someone-playful_grounded</t>
@@ -12977,7 +12977,7 @@
       </c>
       <c r="T128" s="6" t="inlineStr">
         <is>
-          <t>Uỷ quyền 26/10: viết lại → Bạn nói thật lòng một câu, người này cũng đáp lại cởi mở hơn: kết nối không cần kịch bản, chỉ cần bớt chỉnh filter. (Khẳng định cảm xúc người kia không rào: “đáp lại bằng thiện cảm”; đổi sang hành vi thấy được.). Codex chuốt trước khi wiring</t>
+          <t xml:space="preserve">Uỷ quyền 26/10: viết lại → Bạn bỏ bản nháp thứ năm, gửi một câu thật lòng, người này cũng kể thêm: cuộc chat hôm nay bớt một biên tập viên. | Codex chuốt 26/10; Claude review trước khi wiring.</t>
         </is>
       </c>
     </row>
@@ -13077,7 +13077,7 @@
         </is>
       </c>
     </row>
-    <row r="130">
+    <row r="130" ht="60" customHeight="1">
       <c r="A130" s="4" t="inlineStr">
         <is>
           <t>R03-venus-square-jupiter-crush-straight_warm</t>
@@ -13169,7 +13169,7 @@
       </c>
       <c r="T130" s="6" t="inlineStr">
         <is>
-          <t>Uỷ quyền 26/10: viết lại → Khi bạn thể hiện quan tâm vừa phải, crush có thể đáp lại bằng những dự định lớn; hỏi thử một bước cụ thể hai bạn làm được trong tuần này. (Bản cũ ngầm cảnh báo crush không đáng tin). Codex chuốt trước khi wiring</t>
+          <t xml:space="preserve">Uỷ quyền 26/10: viết lại → Khi bạn quan tâm vừa phải, crush có thể nhắc những dự định lớn; hỏi một bước cụ thể hai bạn làm được tuần này. | Codex chuốt 26/10; Claude review trước khi wiring.</t>
         </is>
       </c>
     </row>
@@ -15573,7 +15573,7 @@
         </is>
       </c>
     </row>
-    <row r="156">
+    <row r="156" ht="60" customHeight="1">
       <c r="A156" s="4" t="inlineStr">
         <is>
           <t>R03-moon-square-mars-partner-playful_grounded</t>
@@ -15665,7 +15665,7 @@
       </c>
       <c r="T156" s="6" t="inlineStr">
         <is>
-          <t>Uỷ quyền 26/10: viết lại → Người yêu xắn tay dọn nhà như đánh trận, bạn thì đang cần một cái ôm: chỉ lệch giờ thôi, hẹn lại ca ôm sau khi dọn xong. (Phán xét ngầm: “sai giờ chứ không sai người” ngụ ý “đúng người” (verdict/định mệnh).). Codex chuốt trước khi wiring</t>
+          <t xml:space="preserve">Uỷ quyền 26/10: viết lại → Người yêu đang dọn nhà, bạn lại đứng chờ ôm: gửi yêu cầu đúng lúc máy hút bụi nghỉ giải lao nhé. | Codex chuốt 26/10; Claude review trước khi wiring.</t>
         </is>
       </c>
     </row>
@@ -16341,7 +16341,7 @@
         </is>
       </c>
     </row>
-    <row r="164">
+    <row r="164" ht="60" customHeight="1">
       <c r="A164" s="4" t="inlineStr">
         <is>
           <t>R03-moon-trine-mars-crush-playful_grounded</t>
@@ -16433,7 +16433,7 @@
       </c>
       <c r="T164" s="6" t="inlineStr">
         <is>
-          <t>Uỷ quyền 26/10: viết lại → Bạn đăng story mưa buồn, crush nhắn rủ đi ăn lẩu: phản xạ khá nhanh nhạy, để ý thêm vài lần nữa rồi tính. (Ẩn dụ chấm điểm: “chấm thêm vài lần” là chấm điểm người kia, đi ngược quy tắc không điểm.). Codex chuốt trước khi wiring</t>
+          <t xml:space="preserve">Uỷ quyền 26/10: viết lại → Bạn đăng story mưa buồn, crush rủ ăn lẩu: lòng đã ấm chưa thì chưa biết, nồi lẩu trước mắt có vẻ được. | Codex chuốt 26/10; Claude review trước khi wiring.</t>
         </is>
       </c>
     </row>
@@ -17109,7 +17109,7 @@
         </is>
       </c>
     </row>
-    <row r="172">
+    <row r="172" ht="60" customHeight="1">
       <c r="A172" s="4" t="inlineStr">
         <is>
           <t>R03-moon-trine-mars-partner-playful_grounded</t>
@@ -17201,7 +17201,7 @@
       </c>
       <c r="T172" s="6" t="inlineStr">
         <is>
-          <t>Uỷ quyền 26/10: viết lại → Bạn thở dài một tiếng, người yêu đã dắt xe đi mua cháo: nhanh hơn cả app giao đồ, nhớ cảm ơn bằng lời. (Ẩn dụ chấm điểm: “đánh giá năm sao”; khung “hệ thống …” lặp 4 lần trong playful_grounded.). Codex chuốt trước khi wiring</t>
+          <t xml:space="preserve">Uỷ quyền 26/10: viết lại → Bạn thở dài, người yêu hỏi có cần mua cháo không: chưa kịp mở app giao đồ, nhớ nói mình cần gì nhé. | Codex chuốt 26/10; Claude review trước khi wiring.</t>
         </is>
       </c>
     </row>
@@ -20853,7 +20853,7 @@
         </is>
       </c>
     </row>
-    <row r="211">
+    <row r="211" ht="48" customHeight="1">
       <c r="A211" s="4" t="inlineStr">
         <is>
           <t>R03-venus-trine-sun-crush-gentle_specific</t>
@@ -20945,7 +20945,7 @@
       </c>
       <c r="T211" s="6" t="inlineStr">
         <is>
-          <t>Uỷ quyền 26/10: viết lại → Có thể cách bạn quan tâm sẽ chạm đúng điều crush hay kể về mình; để ý phản hồi thật của họ sau lời khen. (Đoán ý người kia: “chỗ crush muốn được nhìn thấy” gán nhu cầu bên trong.). Codex chuốt trước khi wiring</t>
+          <t xml:space="preserve">Uỷ quyền 26/10: viết lại → Có thể lời khen về điều crush hay kể làm cuộc chat cởi mở hơn; để ý cách họ đáp qua vài lần. | Codex chuốt 26/10; Claude review trước khi wiring.</t>
         </is>
       </c>
     </row>
@@ -22101,7 +22101,7 @@
         </is>
       </c>
     </row>
-    <row r="224">
+    <row r="224" ht="60" customHeight="1">
       <c r="A224" s="4" t="inlineStr">
         <is>
           <t>R03-venus-trine-sun-someone-playful_grounded</t>
@@ -22193,7 +22193,7 @@
       </c>
       <c r="T224" s="6" t="inlineStr">
         <is>
-          <t>Uỷ quyền 26/10: viết lại → Một lời khen đúng chỗ của bạn làm buổi làm quen bớt gượng hẳn: chất xúc tác giao tiếp, không có tác dụng phụ. (“dầu bôi trơn” dễ gợi nghĩa tình dục trong tiếng Việt; lệch ngữ cảnh someone (đồng nghiệp, mới quen).). Codex chuốt trước khi wiring</t>
+          <t xml:space="preserve">Uỷ quyền 26/10: viết lại → Bạn khen đúng chi tiết người này vừa kể, cuộc nói chuyện bớt gượng: lời khen không cần chạy thử mười bản. | Codex chuốt 26/10; Claude review trước khi wiring.</t>
         </is>
       </c>
     </row>
@@ -23925,7 +23925,7 @@
         </is>
       </c>
     </row>
-    <row r="243">
+    <row r="243" ht="48" customHeight="1">
       <c r="A243" s="4" t="inlineStr">
         <is>
           <t>R03-mars-square-mercury-crush-gentle_specific</t>
@@ -24017,7 +24017,7 @@
       </c>
       <c r="T243" s="6" t="inlineStr">
         <is>
-          <t>Uỷ quyền 26/10: viết lại → Có thể sự nôn nóng của bạn gặp lúc crush còn đang hỏi kỹ để cân nhắc; để họ nói hết rồi hãy đề nghị tiếp. (Câu lủng củng: “chạm vào cách crush cần cân nhắc bằng lời” khó hiểu và gán nhu cầu.). Codex chuốt trước khi wiring</t>
+          <t xml:space="preserve">Uỷ quyền 26/10: viết lại → Nếu bạn muốn chốt nhanh lúc crush còn hỏi kỹ, để họ nói hết rồi mới đề nghị bước tiếp theo. | Codex chuốt 26/10; Claude review trước khi wiring.</t>
         </is>
       </c>
     </row>
@@ -29013,7 +29013,7 @@
         </is>
       </c>
     </row>
-    <row r="296">
+    <row r="296" ht="48" customHeight="1">
       <c r="A296" s="4" t="inlineStr">
         <is>
           <t>R03-mercury-conjunction-venus-friend-playful_grounded</t>
@@ -29105,7 +29105,7 @@
       </c>
       <c r="T296" s="6" t="inlineStr">
         <is>
-          <t>Uỷ quyền 26/10: viết lại → Hai đứa có thể nói về một quán bánh suốt hai tiếng: chưa ăn mà đã no vì bàn tán. (Lặp khung: “hội … không lương” (cả hai khung lặp cùng lúc).). Codex chuốt trước khi wiring</t>
+          <t xml:space="preserve">Uỷ quyền 26/10: viết lại → Hai đứa bàn về quán bánh suốt hai tiếng: chưa ăn miếng nào mà thực đơn đã thuộc lòng. | Codex chuốt 26/10; Claude review trước khi wiring.</t>
         </is>
       </c>
     </row>
@@ -30453,7 +30453,7 @@
         </is>
       </c>
     </row>
-    <row r="311">
+    <row r="311" ht="60" customHeight="1">
       <c r="A311" s="4" t="inlineStr">
         <is>
           <t>R03-mercury-opposition-sun-friend-gentle_specific</t>
@@ -30545,7 +30545,7 @@
       </c>
       <c r="T311" s="6" t="inlineStr">
         <is>
-          <t>Uỷ quyền 26/10: viết lại → Lời bạn nói có thể chạm vào một mặt bạn ấy ít khi nhắc tới; chọn lúc riêng tư và hỏi bạn ấy có muốn nghe không. (Đoán nội tâm: “một mặt bạn ấy chưa muốn nhìn” khẳng định bạn ấy đang né tránh.). Codex chuốt trước khi wiring</t>
+          <t xml:space="preserve">Uỷ quyền 26/10: viết lại → Nếu lời bạn định nói liên quan chuyện bạn ấy ít nhắc tới, chọn lúc riêng tư và hỏi họ có muốn nghe không. | Codex chuốt 26/10; Claude review trước khi wiring.</t>
         </is>
       </c>
     </row>
@@ -30933,7 +30933,7 @@
         </is>
       </c>
     </row>
-    <row r="316">
+    <row r="316" ht="60" customHeight="1">
       <c r="A316" s="4" t="inlineStr">
         <is>
           <t>R03-mercury-opposition-sun-partner-playful_grounded</t>
@@ -31025,7 +31025,7 @@
       </c>
       <c r="T316" s="6" t="inlineStr">
         <is>
-          <t>Uỷ quyền 26/10: viết lại → Người yêu bảo năm nay sẽ tiết kiệm, bạn kể ngay ba đơn hàng tháng trước: trí nhớ kiểm toán viên, sắc mà hơi lạnh. (“mở lịch sử chuyển khoản ra đối chiếu” bình thường hóa việc soi giao dịch của người yêu, lệch giá trị riêng tư/tôn trọng của app.). Codex chuốt trước khi wiring</t>
+          <t xml:space="preserve">Uỷ quyền 26/10: viết lại → Người yêu vừa kể kế hoạch tiết kiệm, bạn đã nhớ ba lần cả hai đặt đồ: xin phép góp ý trước khi mở phiên kiểm toán. | Codex chuốt 26/10; Claude review trước khi wiring.</t>
         </is>
       </c>
     </row>
@@ -32853,7 +32853,7 @@
         </is>
       </c>
     </row>
-    <row r="336">
+    <row r="336" ht="60" customHeight="1">
       <c r="A336" s="4" t="inlineStr">
         <is>
           <t>R03-moon-opposition-sun-someone-playful_grounded</t>
@@ -32945,7 +32945,7 @@
       </c>
       <c r="T336" s="6" t="inlineStr">
         <is>
-          <t>Uỷ quyền 26/10: viết lại → Người này là sân khấu, bạn là phòng chờ: không cần đổi chỗ, chỉ cần biết lúc nào mình nên về nghỉ. (“lúc nào nên tắt đèn” mơ hồ, không rõ hành động và có thể gợi nghĩa thân mật với người mới quen.). Codex chuốt trước khi wiring</t>
+          <t xml:space="preserve">Uỷ quyền 26/10: viết lại → Buổi gặp đông người, bạn đã cạn pin mà vẫn ngồi nghe hết chuyện: hôm nay được phép về trước phần hỏi đáp. | Codex chuốt 26/10; Claude review trước khi wiring.</t>
         </is>
       </c>
     </row>
@@ -34389,7 +34389,7 @@
         </is>
       </c>
     </row>
-    <row r="352">
+    <row r="352" ht="60" customHeight="1">
       <c r="A352" s="4" t="inlineStr">
         <is>
           <t>R03-moon-sextile-mercury-someone-playful_grounded</t>
@@ -34481,7 +34481,7 @@
       </c>
       <c r="T352" s="6" t="inlineStr">
         <is>
-          <t>Uỷ quyền 26/10: viết lại → Bạn buột miệng kể hôm nay mệt, người này kể lại chuyện mệt của họ: chưa thân lắm mà đã có chung chủ đề than thở. (Lặp khung: “hội … có N thành viên” (5 lần).). Codex chuốt trước khi wiring</t>
+          <t xml:space="preserve">Uỷ quyền 26/10: viết lại → Bạn vừa than mệt, người này cũng kể ngày dài của họ: chưa thân lắm, đã chung một chủ đề để nghỉ giải lao. | Codex chuốt 26/10; Claude review trước khi wiring.</t>
         </is>
       </c>
     </row>
@@ -34773,7 +34773,7 @@
         </is>
       </c>
     </row>
-    <row r="356">
+    <row r="356" ht="60" customHeight="1">
       <c r="A356" s="4" t="inlineStr">
         <is>
           <t>R03-moon-square-moon-crush-playful_grounded</t>
@@ -34865,7 +34865,7 @@
       </c>
       <c r="T356" s="6" t="inlineStr">
         <is>
-          <t>Uỷ quyền 26/10: viết lại → Bạn buồn thì muốn tâm sự, crush buồn có khi lại lặn mất: hai hệ điều hành cảm xúc, cần cài thêm bộ chuyển đổi. (Đoán ý người kia như sự thật: “crush buồn thì muốn biến mất”; thêm rào “có khi” và đổi sang hành vi.). Codex chuốt trước khi wiring</t>
+          <t xml:space="preserve">Uỷ quyền 26/10: viết lại → Bạn buồn thì nhắn dài, crush có khi im một lúc: khung chat chưa kèm phụ đề, hỏi trước khi tự dịch nhé. | Codex chuốt 26/10; Claude review trước khi wiring.</t>
         </is>
       </c>
     </row>
@@ -38997,7 +38997,7 @@
         </is>
       </c>
     </row>
-    <row r="400">
+    <row r="400" ht="60" customHeight="1">
       <c r="A400" s="4" t="inlineStr">
         <is>
           <t>R03-sun-conjunction-venus-someone-playful_grounded</t>
@@ -39089,7 +39089,7 @@
       </c>
       <c r="T400" s="6" t="inlineStr">
         <is>
-          <t>Uỷ quyền 26/10: viết lại → Bạn nói chuyện như thường ngày, người này cười nhiều hơn dự kiến: đôi khi bớt chuẩn bị lại là chuẩn bị tốt nhất. (Lặp khung: punchline gần trùng dòng crush cùng contact (“chế độ bình thường của bạn đã đủ thú vị” / “phiên bản mặc định khá được”).). Codex chuốt trước khi wiring</t>
+          <t xml:space="preserve">Uỷ quyền 26/10: viết lại → Bạn thôi tập câu mở đầu mà người này lại cười nhiều hơn: hôm nay bản không diễn tập cũng có đất dùng. | Codex chuốt 26/10; Claude review trước khi wiring.</t>
         </is>
       </c>
     </row>
@@ -45141,7 +45141,7 @@
         </is>
       </c>
     </row>
-    <row r="464">
+    <row r="464" ht="60" customHeight="1">
       <c r="A464" s="4" t="inlineStr">
         <is>
           <t>R03-venus-trine-mercury-someone-playful_grounded</t>
@@ -45233,7 +45233,7 @@
       </c>
       <c r="T464" s="6" t="inlineStr">
         <is>
-          <t>Uỷ quyền 26/10: viết lại → Bạn hỏi thêm một câu về điều người này vừa nói, họ hào hứng giải thích cả buổi: câu hỏi đúng chỗ mở được nhiều cửa. (Lặp kịch bản: gần trùng jupiter-trine-sun-someone-playful (khen ý → họ nói thêm nhiều ý); khung “hệ thống …” lặp.). Codex chuốt trước khi wiring</t>
+          <t xml:space="preserve">Uỷ quyền 26/10: viết lại → Bạn hỏi thêm một câu, người này kể cả buổi: phần hỏi đáp dài hơn dự kiến, nhớ chừa lượt cho mình. | Codex chuốt 26/10; Claude review trước khi wiring.</t>
         </is>
       </c>
     </row>
@@ -45717,7 +45717,7 @@
         </is>
       </c>
     </row>
-    <row r="470">
+    <row r="470" ht="60" customHeight="1">
       <c r="A470" s="4" t="inlineStr">
         <is>
           <t>R03-moon-trine-moon-friend-straight_warm</t>
@@ -45809,7 +45809,7 @@
       </c>
       <c r="T470" s="6" t="inlineStr">
         <is>
-          <t>Uỷ quyền 26/10: viết lại → Bạn và bạn ấy dễ cần những thứ giống nhau khi mệt và chăm nhau theo cùng một kiểu; những buổi ngồi không bên nhau cũng quý. (Không tự nhiên: “cùng kiểu cần” thiếu tân ngữ.). Codex chuốt trước khi wiring</t>
+          <t xml:space="preserve">Uỷ quyền 26/10: viết lại → Nếu bạn và bạn ấy hay chọn cùng cách nghỉ khi mệt, những buổi ngồi yên bên nhau cũng đáng giữ; vẫn hỏi xem ai cần gì. | Codex chuốt 26/10; Claude review trước khi wiring.</t>
         </is>
       </c>
     </row>
@@ -47637,7 +47637,7 @@
         </is>
       </c>
     </row>
-    <row r="490">
+    <row r="490" ht="60" customHeight="1">
       <c r="A490" s="4" t="inlineStr">
         <is>
           <t>R03-venus-square-mars-partner-straight_warm</t>
@@ -47729,7 +47729,7 @@
       </c>
       <c r="T490" s="6" t="inlineStr">
         <is>
-          <t>Uỷ quyền 26/10: viết lại → Khi bạn muốn một tối nhẹ nhàng bên nhau mà người yêu đang hừng hực muốn ra ngoài, hai nhịp dễ lệch; nói rõ bạn đang cần gì. (“muốn gần gũi nhẹ nhàng” + “hừng hực năng lượng” (Kim–Hỏa, partner) dễ đọc thành ẩn ý tình dục; làm rõ cảnh đời thường.). Codex chuốt trước khi wiring</t>
+          <t xml:space="preserve">Uỷ quyền 26/10: viết lại → Khi bạn muốn tối yên bên nhau mà người yêu rủ ra ngoài, hai người có thể lệch ý; nói rõ bạn cần gì hôm nay. | Codex chuốt 26/10; Claude review trước khi wiring.</t>
         </is>
       </c>
     </row>
@@ -48213,7 +48213,7 @@
         </is>
       </c>
     </row>
-    <row r="496">
+    <row r="496" ht="60" customHeight="1">
       <c r="A496" s="4" t="inlineStr">
         <is>
           <t>R03-venus-square-mars-someone-playful_grounded</t>
@@ -48305,7 +48305,7 @@
       </c>
       <c r="T496" s="6" t="inlineStr">
         <is>
-          <t>Uỷ quyền 26/10: viết lại → Bạn cười chào xã giao, người này đã gửi kết bạn trên ba mạng: hai bên đang chạy hai tốc độ khác nhau. (Bản cũ nói người kia hiểu bạn thế nào (đoán ý)). Codex chuốt trước khi wiring</t>
+          <t xml:space="preserve">Uỷ quyền 26/10: viết lại → Bạn cười chào xã giao, người này gửi kết bạn ba mạng: khoan bật đủ thông báo, bạn được chọn nhịp của mình. | Codex chuốt 26/10; Claude review trước khi wiring.</t>
         </is>
       </c>
     </row>
@@ -50133,7 +50133,7 @@
         </is>
       </c>
     </row>
-    <row r="516">
+    <row r="516" ht="60" customHeight="1">
       <c r="A516" s="4" t="inlineStr">
         <is>
           <t>R03-neptune-trine-venus-crush-playful_grounded</t>
@@ -50225,7 +50225,7 @@
       </c>
       <c r="T516" s="6" t="inlineStr">
         <is>
-          <t>Uỷ quyền 26/10: viết lại → Bạn gửi một playlist mộng mơ, crush gửi lại một playlist khác: cuộc trò chuyện bằng nhạc vừa mở màn, nghe tiếp xem sao. (Lặp khung: “hội … có N thành viên” xuất hiện 5 lần; bản sửa thêm lời mời quan sát.). Codex chuốt trước khi wiring</t>
+          <t xml:space="preserve">Uỷ quyền 26/10: viết lại → Bạn gửi playlist mộng mơ, crush gửi lại một playlist khác: cuộc chat bằng nhạc đã mở, đừng tự thêm lời tỏ tình. | Codex chuốt 26/10; Claude review trước khi wiring.</t>
         </is>
       </c>
     </row>
@@ -51957,7 +51957,7 @@
         </is>
       </c>
     </row>
-    <row r="535">
+    <row r="535" ht="48" customHeight="1">
       <c r="A535" s="4" t="inlineStr">
         <is>
           <t>R03-sun-conjunction-true_node-friend-gentle_specific</t>
@@ -52049,11 +52049,11 @@
       </c>
       <c r="T535" s="6" t="inlineStr">
         <is>
-          <t>Uỷ quyền 26/10: viết lại → Có thể bạn ấy hay để ý cách bạn tự tin xử lý mọi việc; ở bên và khích lệ khi bạn ấy thử là đủ. (Đoán nội tâm, hơi bề trên: “sự tự tin của bạn là điều bạn ấy đang tập” khẳng định điểm yếu của bạn ấy.). Codex chuốt trước khi wiring</t>
-        </is>
-      </c>
-    </row>
-    <row r="536">
+          <t xml:space="preserve">Uỷ quyền 26/10: viết lại → Lúc bạn ấy hỏi cách bạn làm rồi thử theo, chia sẻ phần hữu ích và để bạn ấy tự chọn cách riêng. | Codex chuốt 26/10; Claude review trước khi wiring.</t>
+        </is>
+      </c>
+    </row>
+    <row r="536" ht="48" customHeight="1">
       <c r="A536" s="4" t="inlineStr">
         <is>
           <t>R03-sun-conjunction-true_node-friend-playful_grounded</t>
@@ -52145,7 +52145,7 @@
       </c>
       <c r="T536" s="6" t="inlineStr">
         <is>
-          <t>Uỷ quyền 26/10: viết lại → Thấy bạn đọc sách, bạn ấy cũng ôm về một chồng: thói quen tốt mà lây được thì cứ để nó lây. (Lặp khung: “… không lương / miễn phí / không thu phí” xuất hiện 5 lần.). Codex chuốt trước khi wiring</t>
+          <t xml:space="preserve">Uỷ quyền 26/10: viết lại → Thấy bạn đọc sách, bạn ấy cũng ôm về một chồng: hội đọc chưa họp, danh sách mượn đã dài. | Codex chuốt 26/10; Claude review trước khi wiring.</t>
         </is>
       </c>
     </row>
@@ -53877,7 +53877,7 @@
         </is>
       </c>
     </row>
-    <row r="555">
+    <row r="555" ht="60" customHeight="1">
       <c r="A555" s="4" t="inlineStr">
         <is>
           <t>R03-sun-conjunction-uranus-partner-gentle_specific</t>
@@ -53969,7 +53969,7 @@
       </c>
       <c r="T555" s="6" t="inlineStr">
         <is>
-          <t>Uỷ quyền 26/10: viết lại → Có thể những lần người yêu muốn đổi mới nếp sống lại chạm vào chỗ bạn cần ổn định; nói rõ điều gì cần giữ nguyên. (Gán nhu cầu (“nhu cầu tự do của người yêu”) và tối nghĩa (“được nhìn nhận ổn định”).). Codex chuốt trước khi wiring</t>
+          <t xml:space="preserve">Uỷ quyền 26/10: viết lại → Nếu người yêu đề nghị đổi nếp sống lúc bạn cần ổn định, nói rõ điều bạn muốn giữ trước khi bàn phần thay đổi. | Codex chuốt 26/10; Claude review trước khi wiring.</t>
         </is>
       </c>
     </row>
@@ -54807,7 +54807,7 @@
         </is>
       </c>
     </row>
-    <row r="6">
+    <row r="6" ht="26.399999618530273" customHeight="1">
       <c r="A6" s="9" t="inlineStr">
         <is>
           <t>R03-true_node-square-sun-crush-deep_dive</t>
@@ -54835,11 +54835,11 @@
       </c>
       <c r="F6" s="9" t="inlineStr">
         <is>
-          <t>Cách crush sống sôi nổi đôi khi làm bạn chao đảo với hướng mới đang tập, nên ghi lại lý do mình bắt đầu rồi xem sau vài lần gặp nó còn vững không.</t>
-        </is>
-      </c>
-      <c r="G6" s="9" t="n">
-        <v>34</v>
+          <t xml:space="preserve">Nếu lời rủ của crush làm bạn lưỡng lự với nếp mới đang tập, ghi lại điều mình muốn giữ rồi nói rõ, vì bạn không cần đổi hướng chỉ để theo kịp người khác.</t>
+        </is>
+      </c>
+      <c r="G6" s="9">
+        <v>35</v>
       </c>
       <c r="H6" s="9" t="inlineStr">
         <is>
@@ -54848,7 +54848,7 @@
       </c>
       <c r="I6" s="9" t="inlineStr">
         <is>
-          <t>Uỷ quyền 26/10: duyệt bản nháp (giọng deep_dive cho phép tối đa 40 âm tiết). Codex chuốt trước khi wiring; cần chuốt: câu dễ cấn hơi nghiêng về mô tả người kia hoặc ngầm hứa tiến triển</t>
+          <t xml:space="preserve">Uỷ quyền 26/10: duyệt bản nháp; Codex chuốt 26/10 để giữ tình huống có điều kiện, không giả định lịch sử gặp hay ý người kia. Claude review trước khi wiring.</t>
         </is>
       </c>
     </row>
@@ -54942,7 +54942,7 @@
         </is>
       </c>
     </row>
-    <row r="9">
+    <row r="9" ht="26.399999618530273" customHeight="1">
       <c r="A9" s="9" t="inlineStr">
         <is>
           <t>R03-true_node-square-sun-someone-deep_dive</t>
@@ -54970,10 +54970,10 @@
       </c>
       <c r="F9" s="9" t="inlineStr">
         <is>
-          <t>Thứ hiện ra rõ nhất là giọng chắc nịch của người này đôi khi làm bạn lung lay; dùng lúc đó để hỏi lại hướng của mình, vì người khác không quyết thay bạn.</t>
-        </is>
-      </c>
-      <c r="G9" s="9" t="n">
+          <t xml:space="preserve">Nếu bạn đổi ý ngay sau khi nghe người này trình bày, dành lúc riêng xem lại lý do ban đầu, vì giọng nói tự tin chưa đủ để quyết thay điều bạn chọn.</t>
+        </is>
+      </c>
+      <c r="G9" s="9">
         <v>34</v>
       </c>
       <c r="H9" s="9" t="inlineStr">
@@ -54983,7 +54983,7 @@
       </c>
       <c r="I9" s="9" t="inlineStr">
         <is>
-          <t>Uỷ quyền 26/10: duyệt bản nháp (giọng deep_dive cho phép tối đa 40 âm tiết). Codex chuốt trước khi wiring; cần chuốt: câu dễ cấn hơi nghiêng về mô tả người kia hoặc ngầm hứa tiến triển</t>
+          <t xml:space="preserve">Uỷ quyền 26/10: duyệt bản nháp; Codex chuốt 26/10 để giữ tình huống có điều kiện, không giả định lịch sử gặp hay ý người kia. Claude review trước khi wiring.</t>
         </is>
       </c>
     </row>
@@ -55077,7 +55077,7 @@
         </is>
       </c>
     </row>
-    <row r="12">
+    <row r="12" ht="26.399999618530273" customHeight="1">
       <c r="A12" s="9" t="inlineStr">
         <is>
           <t>R03-jupiter-trine-pluto-partner-deep_dive</t>
@@ -55105,11 +55105,11 @@
       </c>
       <c r="F12" s="9" t="inlineStr">
         <is>
-          <t>Một mẫu hay lặp lại là người yêu nói ra nỗi lo sâu nhất vào những tối bạn giữ giọng bình tĩnh; ghi nhận trước khi động viên, rồi đối chiếu qua vài tuần.</t>
-        </is>
-      </c>
-      <c r="G12" s="9" t="n">
-        <v>34</v>
+          <t xml:space="preserve">Nếu người yêu kể chuyện lo lắng lúc bạn giữ giọng bình tĩnh, ghi nhận trước khi động viên rồi hỏi họ cần gì, vì một lần nói chuyện chưa cho biết cách nào luôn phù hợp.</t>
+        </is>
+      </c>
+      <c r="G12" s="9">
+        <v>37</v>
       </c>
       <c r="H12" s="9" t="inlineStr">
         <is>
@@ -55118,7 +55118,7 @@
       </c>
       <c r="I12" s="9" t="inlineStr">
         <is>
-          <t>Uỷ quyền 26/10: duyệt bản nháp (giọng deep_dive cho phép tối đa 40 âm tiết). Codex chuốt trước khi wiring</t>
+          <t xml:space="preserve">Uỷ quyền 26/10: duyệt bản nháp; Codex chuốt 26/10 để giữ tình huống có điều kiện, không giả định lịch sử gặp hay ý người kia. Claude review trước khi wiring.</t>
         </is>
       </c>
     </row>
@@ -55212,7 +55212,7 @@
         </is>
       </c>
     </row>
-    <row r="15">
+    <row r="15" ht="26.399999618530273" customHeight="1">
       <c r="A15" s="9" t="inlineStr">
         <is>
           <t>R03-jupiter-trine-sun-friend-deep_dive</t>
@@ -55240,11 +55240,11 @@
       </c>
       <c r="F15" s="9" t="inlineStr">
         <is>
-          <t>Bạn thường nhận vai người cổ vũ sớm nhất mỗi lần bạn ấy cân nhắc một bước ngoặt; hỏi xem kiểu cổ vũ nào giúp được bạn ấy thật, thay vì đoán.</t>
-        </is>
-      </c>
-      <c r="G15" s="9" t="n">
-        <v>32</v>
+          <t xml:space="preserve">Trước một bước ngoặt của bạn ấy, bạn có thể hỏi muốn được lắng nghe hay góp ý rồi mới cổ vũ, vì điều giúp ích là do bạn ấy nói, không phải mình đoán.</t>
+        </is>
+      </c>
+      <c r="G15" s="9">
+        <v>35</v>
       </c>
       <c r="H15" s="9" t="inlineStr">
         <is>
@@ -55253,7 +55253,7 @@
       </c>
       <c r="I15" s="9" t="inlineStr">
         <is>
-          <t>Uỷ quyền 26/10: duyệt bản nháp (giọng deep_dive cho phép tối đa 40 âm tiết). Codex chuốt trước khi wiring</t>
+          <t xml:space="preserve">Uỷ quyền 26/10: duyệt bản nháp; Codex chuốt 26/10 để giữ tình huống có điều kiện, không giả định lịch sử gặp hay ý người kia. Claude review trước khi wiring.</t>
         </is>
       </c>
     </row>
@@ -55482,7 +55482,7 @@
         </is>
       </c>
     </row>
-    <row r="21">
+    <row r="21" ht="26.399999618530273" customHeight="1">
       <c r="A21" s="9" t="inlineStr">
         <is>
           <t>R03-mercury-square-sun-someone-deep_dive</t>
@@ -55510,11 +55510,11 @@
       </c>
       <c r="F21" s="9" t="inlineStr">
         <is>
-          <t>Giữa bạn và người này, câu hỏi vặn đôi khi bật ra ngay lúc họ kể điều mình làm được; mở bằng một lời ghi nhận, rồi để ý không khí buổi trao đổi thay đổi ra sao.</t>
-        </is>
-      </c>
-      <c r="G21" s="9" t="n">
-        <v>38</v>
+          <t xml:space="preserve">Nếu bạn hỏi dồn lúc người này vừa kể thành quả, ghi nhận một việc cụ thể trước khi hỏi thêm, rồi để ý họ đáp ra sao thay vì tự đoán ý sau vẻ mặt.</t>
+        </is>
+      </c>
+      <c r="G21" s="9">
+        <v>36</v>
       </c>
       <c r="H21" s="9" t="inlineStr">
         <is>
@@ -55523,7 +55523,7 @@
       </c>
       <c r="I21" s="9" t="inlineStr">
         <is>
-          <t>Uỷ quyền 26/10: duyệt bản nháp (giọng deep_dive cho phép tối đa 40 âm tiết). Codex chuốt trước khi wiring</t>
+          <t xml:space="preserve">Uỷ quyền 26/10: duyệt bản nháp; Codex chuốt 26/10 để giữ tình huống có điều kiện, không giả định lịch sử gặp hay ý người kia. Claude review trước khi wiring.</t>
         </is>
       </c>
     </row>
@@ -55617,7 +55617,7 @@
         </is>
       </c>
     </row>
-    <row r="24">
+    <row r="24" ht="26.399999618530273" customHeight="1">
       <c r="A24" s="9" t="inlineStr">
         <is>
           <t>R03-mercury-trine-true_node-partner-deep_dive</t>
@@ -55645,11 +55645,11 @@
       </c>
       <c r="F24" s="9" t="inlineStr">
         <is>
-          <t>Trong những bữa tối, câu hỏi bạn đặt ra dễ giúp người yêu vạch rõ bước tiếp theo; để họ tự trả lời, rồi xem hướng đó có thành hình qua vài tháng.</t>
-        </is>
-      </c>
-      <c r="G24" s="9" t="n">
-        <v>33</v>
+          <t xml:space="preserve">Nếu câu hỏi của bạn giúp người yêu nói rõ việc tiếp theo, để họ tự chọn bước muốn làm và hỏi lại khi họ nhắc tới, vì nói được chưa có nghĩa là đã quyết.</t>
+        </is>
+      </c>
+      <c r="G24" s="9">
+        <v>36</v>
       </c>
       <c r="H24" s="9" t="inlineStr">
         <is>
@@ -55658,7 +55658,7 @@
       </c>
       <c r="I24" s="9" t="inlineStr">
         <is>
-          <t>Uỷ quyền 26/10: duyệt bản nháp (giọng deep_dive cho phép tối đa 40 âm tiết). Codex chuốt trước khi wiring</t>
+          <t xml:space="preserve">Uỷ quyền 26/10: duyệt bản nháp; Codex chuốt 26/10 để giữ tình huống có điều kiện, không giả định lịch sử gặp hay ý người kia. Claude review trước khi wiring.</t>
         </is>
       </c>
     </row>
@@ -55977,7 +55977,7 @@
         </is>
       </c>
     </row>
-    <row r="32">
+    <row r="32" ht="26.399999618530273" customHeight="1">
       <c r="A32" s="9" t="inlineStr">
         <is>
           <t>R03-sun-trine-venus-partner-deep_dive</t>
@@ -56005,11 +56005,11 @@
       </c>
       <c r="F32" s="9" t="inlineStr">
         <is>
-          <t>Nhìn qua nhiều ngày, những hôm bạn tự tin làm việc mình giỏi thường đi cùng cử chỉ chăm sóc của người yêu; gọi tên cử chỉ đó, nhưng không cần phải giỏi mới được chăm.</t>
-        </is>
-      </c>
-      <c r="G32" s="9" t="n">
-        <v>36</v>
+          <t xml:space="preserve">Nếu bạn nhận thấy người yêu quan tâm khi mình kể việc làm tốt, ghi nhận cử chỉ cụ thể ấy và nói điều bạn cần, vì bạn không cần giỏi mới xứng đáng được quan tâm.</t>
+        </is>
+      </c>
+      <c r="G32" s="9">
+        <v>37</v>
       </c>
       <c r="H32" s="9" t="inlineStr">
         <is>
@@ -56018,7 +56018,7 @@
       </c>
       <c r="I32" s="9" t="inlineStr">
         <is>
-          <t>Uỷ quyền 26/10: duyệt bản nháp (giọng deep_dive cho phép tối đa 40 âm tiết). Codex chuốt trước khi wiring</t>
+          <t xml:space="preserve">Uỷ quyền 26/10: duyệt bản nháp; Codex chuốt 26/10 để giữ tình huống có điều kiện, không giả định lịch sử gặp hay ý người kia. Claude review trước khi wiring.</t>
         </is>
       </c>
     </row>
@@ -56202,7 +56202,7 @@
         </is>
       </c>
     </row>
-    <row r="37">
+    <row r="37" ht="26.399999618530273" customHeight="1">
       <c r="A37" s="9" t="inlineStr">
         <is>
           <t>R03-venus-square-jupiter-someone-deep_dive</t>
@@ -56230,11 +56230,11 @@
       </c>
       <c r="F37" s="9" t="inlineStr">
         <is>
-          <t>Điều cần đọc kỹ là những kế hoạch lớn người này đưa ra ngay lần đầu dễ làm bạn ngợp, nên nhìn vào những gì họ làm sau đó, và bạn được quyền đi chậm.</t>
-        </is>
-      </c>
-      <c r="G37" s="9" t="n">
-        <v>35</v>
+          <t xml:space="preserve">Nếu bạn thấy ngợp khi người này đề nghị những việc lớn ngay lần đầu, nói rõ phần mình sẵn sàng làm rồi quan sát cách họ đáp, vì bạn được quyền chọn mức tham gia.</t>
+        </is>
+      </c>
+      <c r="G37" s="9">
+        <v>36</v>
       </c>
       <c r="H37" s="9" t="inlineStr">
         <is>
@@ -56243,7 +56243,7 @@
       </c>
       <c r="I37" s="9" t="inlineStr">
         <is>
-          <t>Uỷ quyền 26/10: duyệt bản nháp (giọng deep_dive cho phép tối đa 40 âm tiết). Codex chuốt trước khi wiring; cần chuốt: câu dễ cấn hơi nghiêng về mô tả người kia hoặc ngầm hứa tiến triển</t>
+          <t xml:space="preserve">Uỷ quyền 26/10: duyệt bản nháp; Codex chuốt 26/10 để giữ tình huống có điều kiện, không giả định lịch sử gặp hay ý người kia. Claude review trước khi wiring.</t>
         </is>
       </c>
     </row>
@@ -56787,7 +56787,7 @@
         </is>
       </c>
     </row>
-    <row r="50">
+    <row r="50" ht="26.399999618530273" customHeight="1">
       <c r="A50" s="9" t="inlineStr">
         <is>
           <t>R03-venus-trine-mars-crush-deep_dive</t>
@@ -56815,10 +56815,10 @@
       </c>
       <c r="F50" s="9" t="inlineStr">
         <is>
-          <t>Điều lớp này ghi nhận là sự ân cần nhỏ của bạn hay được crush trả lời bằng việc làm, như hẹn một buổi cụ thể; nhìn chuỗi hành động qua vài tuần thay vì một lời mời.</t>
-        </is>
-      </c>
-      <c r="G50" s="9" t="n">
+          <t xml:space="preserve">Nếu bạn quan tâm bằng lời còn crush đáp bằng một lời hẹn cụ thể, đối chiếu thêm những lần sau và giữ nhịp mình thấy thoải mái, vì một lời mời chưa xác định mối quan hệ.</t>
+        </is>
+      </c>
+      <c r="G50" s="9">
         <v>38</v>
       </c>
       <c r="H50" s="9" t="inlineStr">
@@ -56828,7 +56828,7 @@
       </c>
       <c r="I50" s="9" t="inlineStr">
         <is>
-          <t>Uỷ quyền 26/10: duyệt bản nháp (giọng deep_dive cho phép tối đa 40 âm tiết). Codex chuốt trước khi wiring</t>
+          <t xml:space="preserve">Uỷ quyền 26/10: duyệt bản nháp; Codex chuốt 26/10 để giữ tình huống có điều kiện, không giả định lịch sử gặp hay ý người kia. Claude review trước khi wiring.</t>
         </is>
       </c>
     </row>
@@ -56922,7 +56922,7 @@
         </is>
       </c>
     </row>
-    <row r="53">
+    <row r="53" ht="26.399999618530273" customHeight="1">
       <c r="A53" s="9" t="inlineStr">
         <is>
           <t>R03-venus-trine-mars-someone-deep_dive</t>
@@ -56950,10 +56950,10 @@
       </c>
       <c r="F53" s="9" t="inlineStr">
         <is>
-          <t>Một quan sát đáng giữ là sự thân thiện của bạn dễ dẫn tới việc người này đề nghị làm chung một việc; bạn được quyền cân nhắc, vì một lời mời chưa nói lên mức thân.</t>
-        </is>
-      </c>
-      <c r="G53" s="9" t="n">
+          <t xml:space="preserve">Nếu lời bắt chuyện của bạn dẫn tới đề nghị làm chung việc gì đó, cứ hỏi rõ phần mình rồi cân nhắc, vì một lời mời chưa nói lên mức độ thân quen giữa hai người.</t>
+        </is>
+      </c>
+      <c r="G53" s="9">
         <v>37</v>
       </c>
       <c r="H53" s="9" t="inlineStr">
@@ -56963,7 +56963,7 @@
       </c>
       <c r="I53" s="9" t="inlineStr">
         <is>
-          <t>Uỷ quyền 26/10: duyệt bản nháp (giọng deep_dive cho phép tối đa 40 âm tiết). Codex chuốt trước khi wiring</t>
+          <t xml:space="preserve">Uỷ quyền 26/10: duyệt bản nháp; Codex chuốt 26/10 để giữ tình huống có điều kiện, không giả định lịch sử gặp hay ý người kia. Claude review trước khi wiring.</t>
         </is>
       </c>
     </row>
@@ -57012,7 +57012,7 @@
         </is>
       </c>
     </row>
-    <row r="55">
+    <row r="55" ht="26.399999618530273" customHeight="1">
       <c r="A55" s="9" t="inlineStr">
         <is>
           <t>R03-venus-trine-sun-friend-deep_dive</t>
@@ -57040,10 +57040,10 @@
       </c>
       <c r="F55" s="9" t="inlineStr">
         <is>
-          <t>Vai quen của bạn là người ghi nhận khi bạn ấy vượt qua một việc khó, như sau kỳ thi hay buổi ra mắt sản phẩm, nên giữ thói quen nhắn một câu, rồi xem cách bạn ấy đáp.</t>
-        </is>
-      </c>
-      <c r="G55" s="9" t="n">
+          <t xml:space="preserve">Khi bạn ấy kể vừa vượt qua một việc khó, lời ghi nhận cụ thể của bạn có thể mở thêm cuộc trò chuyện, nhưng vẫn hỏi họ có muốn kể tiếp thay vì tự nhận vai động viên.</t>
+        </is>
+      </c>
+      <c r="G55" s="9">
         <v>39</v>
       </c>
       <c r="H55" s="9" t="inlineStr">
@@ -57053,11 +57053,11 @@
       </c>
       <c r="I55" s="9" t="inlineStr">
         <is>
-          <t>Uỷ quyền 26/10: duyệt bản nháp (giọng deep_dive cho phép tối đa 40 âm tiết). Codex chuốt trước khi wiring</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
+          <t xml:space="preserve">Uỷ quyền 26/10: duyệt bản nháp; Codex chuốt 26/10 để giữ tình huống có điều kiện, không giả định lịch sử gặp hay ý người kia. Claude review trước khi wiring.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="26.399999618530273" customHeight="1">
       <c r="A56" s="9" t="inlineStr">
         <is>
           <t>R03-venus-trine-sun-partner-deep_dive</t>
@@ -57085,11 +57085,11 @@
       </c>
       <c r="F56" s="9" t="inlineStr">
         <is>
-          <t>Lớp đầu tiên là một câu cảm ơn có tên việc cụ thể, như “cảm ơn vì đã sửa vòi nước”, thường làm người yêu hăng hái hơn với việc chung; thử một tuần rồi xem nhà mình đổi gì.</t>
-        </is>
-      </c>
-      <c r="G56" s="9" t="n">
-        <v>40</v>
+          <t xml:space="preserve">Một lời cảm ơn gọi tên việc cụ thể, như sửa vòi nước, có thể giúp hai bạn nói rõ sự quan tâm; hỏi người yêu việc nào có ý nghĩa, thay vì tự đánh giá hộ họ.</t>
+        </is>
+      </c>
+      <c r="G56" s="9">
+        <v>38</v>
       </c>
       <c r="H56" s="9" t="inlineStr">
         <is>
@@ -57098,7 +57098,7 @@
       </c>
       <c r="I56" s="9" t="inlineStr">
         <is>
-          <t>Uỷ quyền 26/10: duyệt bản nháp (giọng deep_dive cho phép tối đa 40 âm tiết). Codex chuốt trước khi wiring</t>
+          <t xml:space="preserve">Uỷ quyền 26/10: duyệt bản nháp; Codex chuốt 26/10 để giữ tình huống có điều kiện, không giả định lịch sử gặp hay ý người kia. Claude review trước khi wiring.</t>
         </is>
       </c>
     </row>
@@ -57192,7 +57192,7 @@
         </is>
       </c>
     </row>
-    <row r="59">
+    <row r="59" ht="26.399999618530273" customHeight="1">
       <c r="A59" s="9" t="inlineStr">
         <is>
           <t>R03-mars-sextile-moon-friend-deep_dive</t>
@@ -57220,11 +57220,11 @@
       </c>
       <c r="F59" s="9" t="inlineStr">
         <is>
-          <t>Ở các kèo nhóm, bạn đứng ra lên lịch còn bạn ấy tới với tâm trạng thoải mái, một nhịp khá dễ đi; hỏi ý trước khi chốt, rồi xem bạn ấy có rủ lại không.</t>
-        </is>
-      </c>
-      <c r="G59" s="9" t="n">
-        <v>36</v>
+          <t xml:space="preserve">Khi lên lịch gặp nhóm, bạn có thể hỏi phần nào giúp bạn ấy thoải mái rồi mới chốt; để ý cả những lần họ chủ động rủ lại, vì phối hợp cần lượt của hai người.</t>
+        </is>
+      </c>
+      <c r="G59" s="9">
+        <v>37</v>
       </c>
       <c r="H59" s="9" t="inlineStr">
         <is>
@@ -57233,7 +57233,7 @@
       </c>
       <c r="I59" s="9" t="inlineStr">
         <is>
-          <t>Uỷ quyền 26/10: duyệt bản nháp (giọng deep_dive cho phép tối đa 40 âm tiết). Codex chuốt trước khi wiring</t>
+          <t xml:space="preserve">Uỷ quyền 26/10: duyệt bản nháp; Codex chuốt 26/10 để giữ tình huống có điều kiện, không giả định lịch sử gặp hay ý người kia. Claude review trước khi wiring.</t>
         </is>
       </c>
     </row>
@@ -57552,7 +57552,7 @@
         </is>
       </c>
     </row>
-    <row r="67">
+    <row r="67" ht="26.399999618530273" customHeight="1">
       <c r="A67" s="9" t="inlineStr">
         <is>
           <t>R03-mars-trine-sun-friend-deep_dive</t>
@@ -57580,11 +57580,11 @@
       </c>
       <c r="F67" s="9" t="inlineStr">
         <is>
-          <t>Nhìn qua những thử thách hai đứa từng làm, bạn hay là người rủ còn bạn ấy là người tỏa sáng khi làm, nên để bạn ấy tự nhận phần việc và hỏi lại khi thấy nhịp quá dày.</t>
-        </is>
-      </c>
-      <c r="G67" s="9" t="n">
-        <v>39</v>
+          <t xml:space="preserve">Nếu bạn khởi xướng một việc còn bạn ấy nhận phần làm sở trường, chia rõ phạm vi và hỏi lịch có vừa không, vì làm tốt một lần chưa nói lên cách phối hợp lâu dài.</t>
+        </is>
+      </c>
+      <c r="G67" s="9">
+        <v>37</v>
       </c>
       <c r="H67" s="9" t="inlineStr">
         <is>
@@ -57593,11 +57593,11 @@
       </c>
       <c r="I67" s="9" t="inlineStr">
         <is>
-          <t>Uỷ quyền 26/10: duyệt bản nháp (giọng deep_dive cho phép tối đa 40 âm tiết). Codex chuốt trước khi wiring</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
+          <t xml:space="preserve">Uỷ quyền 26/10: duyệt bản nháp; Codex chuốt 26/10 để giữ tình huống có điều kiện, không giả định lịch sử gặp hay ý người kia. Claude review trước khi wiring.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" ht="26.399999618530273" customHeight="1">
       <c r="A68" s="9" t="inlineStr">
         <is>
           <t>R03-mars-trine-sun-partner-deep_dive</t>
@@ -57625,11 +57625,11 @@
       </c>
       <c r="F68" s="9" t="inlineStr">
         <is>
-          <t>Nhìn theo tuần, kế hoạch bạn khởi xướng như tập thể dục hay nấu món mới thường là chỗ người yêu thể hiện sở trường; luân phiên người khởi xướng, rồi sau một tháng hỏi nhau nhịp có vừa không.</t>
-        </is>
-      </c>
-      <c r="G68" s="9" t="n">
-        <v>40</v>
+          <t xml:space="preserve">Khi bạn rủ tập hay nấu món mới, để người yêu chọn phần họ muốn thử rồi luân phiên khởi xướng; hỏi lại sau vài lần, vì một người luôn lên lịch cũng có thể thấy mệt.</t>
+        </is>
+      </c>
+      <c r="G68" s="9">
+        <v>37</v>
       </c>
       <c r="H68" s="9" t="inlineStr">
         <is>
@@ -57638,7 +57638,7 @@
       </c>
       <c r="I68" s="9" t="inlineStr">
         <is>
-          <t>Uỷ quyền 26/10: duyệt bản nháp (giọng deep_dive cho phép tối đa 40 âm tiết). Codex chuốt trước khi wiring</t>
+          <t xml:space="preserve">Uỷ quyền 26/10: duyệt bản nháp; Codex chuốt 26/10 để giữ tình huống có điều kiện, không giả định lịch sử gặp hay ý người kia. Claude review trước khi wiring.</t>
         </is>
       </c>
     </row>
@@ -57957,7 +57957,7 @@
         </is>
       </c>
     </row>
-    <row r="76">
+    <row r="76" ht="26.399999618530273" customHeight="1">
       <c r="A76" s="9" t="inlineStr">
         <is>
           <t>R03-mercury-conjunction-venus-partner-deep_dive</t>
@@ -57985,11 +57985,11 @@
       </c>
       <c r="F76" s="9" t="inlineStr">
         <is>
-          <t>Theo nếp hằng ngày, những tin nhắn nhỏ kiểu “về cẩn thận nhé” của bạn thường được người yêu nhắc lại vào hôm sau, nên để ý xem chúng có thưa đi vào tuần bận không, rồi tự điều chỉnh.</t>
-        </is>
-      </c>
-      <c r="G76" s="9" t="n">
-        <v>40</v>
+          <t xml:space="preserve">Với những tin nhắn hỏi han hằng ngày, bạn có thể để ý lúc nào người yêu đáp lại và hỏi họ cách nào dễ chịu, vì tuần bận ít tin chưa nói lên mức độ quan tâm.</t>
+        </is>
+      </c>
+      <c r="G76" s="9">
+        <v>38</v>
       </c>
       <c r="H76" s="9" t="inlineStr">
         <is>
@@ -57998,7 +57998,7 @@
       </c>
       <c r="I76" s="9" t="inlineStr">
         <is>
-          <t>Uỷ quyền 26/10: duyệt bản nháp (giọng deep_dive cho phép tối đa 40 âm tiết). Codex chuốt trước khi wiring</t>
+          <t xml:space="preserve">Uỷ quyền 26/10: duyệt bản nháp; Codex chuốt 26/10 để giữ tình huống có điều kiện, không giả định lịch sử gặp hay ý người kia. Claude review trước khi wiring.</t>
         </is>
       </c>
     </row>
@@ -58092,7 +58092,7 @@
         </is>
       </c>
     </row>
-    <row r="79">
+    <row r="79" ht="26.399999618530273" customHeight="1">
       <c r="A79" s="9" t="inlineStr">
         <is>
           <t>R03-mercury-opposition-sun-friend-deep_dive</t>
@@ -58120,11 +58120,11 @@
       </c>
       <c r="F79" s="9" t="inlineStr">
         <is>
-          <t>Trong nhiều buổi cà phê, góc nhìn của bạn về một chuyện thường ngược với cách bạn ấy kể, nên xin phép trước khi phản biện, và để ý không khí giữa hai đứa sau mỗi lần bàn.</t>
-        </is>
-      </c>
-      <c r="G79" s="9" t="n">
-        <v>38</v>
+          <t xml:space="preserve">Nếu cách bạn hiểu một chuyện khác với lời bạn ấy kể, xin phép trước khi góp ý rồi nghe câu trả lời, vì góc nhìn khác không tự động là hiểu rõ người kia hơn.</t>
+        </is>
+      </c>
+      <c r="G79" s="9">
+        <v>36</v>
       </c>
       <c r="H79" s="9" t="inlineStr">
         <is>
@@ -58133,7 +58133,7 @@
       </c>
       <c r="I79" s="9" t="inlineStr">
         <is>
-          <t>Uỷ quyền 26/10: duyệt bản nháp (giọng deep_dive cho phép tối đa 40 âm tiết). Codex chuốt trước khi wiring</t>
+          <t xml:space="preserve">Uỷ quyền 26/10: duyệt bản nháp; Codex chuốt 26/10 để giữ tình huống có điều kiện, không giả định lịch sử gặp hay ý người kia. Claude review trước khi wiring.</t>
         </is>
       </c>
     </row>
@@ -58182,7 +58182,7 @@
         </is>
       </c>
     </row>
-    <row r="81">
+    <row r="81" ht="26.399999618530273" customHeight="1">
       <c r="A81" s="9" t="inlineStr">
         <is>
           <t>R03-mercury-opposition-sun-someone-deep_dive</t>
@@ -58210,10 +58210,10 @@
       </c>
       <c r="F81" s="9" t="inlineStr">
         <is>
-          <t>Ghi nhận đầu tiên là ý kiến của bạn và người này hay đứng ở hai đầu, kể cả trong chuyện nhỏ; để họ nói xong rồi mới đáp, vì khác góc nhìn không phải chuyện đúng sai.</t>
-        </is>
-      </c>
-      <c r="G81" s="9" t="n">
+          <t xml:space="preserve">Nếu bạn và người này nêu hai ý trái nhau, để họ nói hết rồi hỏi lại phần mình chưa rõ trước khi đáp, vì một bất đồng chưa mô tả được cả cách hai người hợp tác.</t>
+        </is>
+      </c>
+      <c r="G81" s="9">
         <v>38</v>
       </c>
       <c r="H81" s="9" t="inlineStr">
@@ -58223,7 +58223,7 @@
       </c>
       <c r="I81" s="9" t="inlineStr">
         <is>
-          <t>Uỷ quyền 26/10: duyệt bản nháp (giọng deep_dive cho phép tối đa 40 âm tiết). Codex chuốt trước khi wiring</t>
+          <t xml:space="preserve">Uỷ quyền 26/10: duyệt bản nháp; Codex chuốt 26/10 để giữ tình huống có điều kiện, không giả định lịch sử gặp hay ý người kia. Claude review trước khi wiring.</t>
         </is>
       </c>
     </row>
@@ -58272,7 +58272,7 @@
         </is>
       </c>
     </row>
-    <row r="83">
+    <row r="83" ht="26.399999618530273" customHeight="1">
       <c r="A83" s="9" t="inlineStr">
         <is>
           <t>R03-moon-opposition-sun-friend-deep_dive</t>
@@ -58300,11 +58300,11 @@
       </c>
       <c r="F83" s="9" t="inlineStr">
         <is>
-          <t>Những tuần bạn ấy bận chạy dự án hay trùng lúc bạn mong một buổi ngồi gần nói chuyện; giữ một lịch cố định mỗi tháng rồi xem hai đứa có đỡ hụt nhau không.</t>
-        </is>
-      </c>
-      <c r="G83" s="9" t="n">
-        <v>35</v>
+          <t xml:space="preserve">Nếu lịch bận của bạn ấy trùng lúc bạn muốn gặp, đề xuất một dịp cụ thể rồi hỏi thời gian nào vừa, vì chưa sắp được một buổi không có nghĩa là tình bạn kém quan trọng.</t>
+        </is>
+      </c>
+      <c r="G83" s="9">
+        <v>38</v>
       </c>
       <c r="H83" s="9" t="inlineStr">
         <is>
@@ -58313,11 +58313,11 @@
       </c>
       <c r="I83" s="9" t="inlineStr">
         <is>
-          <t>Uỷ quyền 26/10: duyệt bản nháp (giọng deep_dive cho phép tối đa 40 âm tiết). Codex chuốt trước khi wiring</t>
-        </is>
-      </c>
-    </row>
-    <row r="84">
+          <t xml:space="preserve">Uỷ quyền 26/10: duyệt bản nháp; Codex chuốt 26/10 để giữ tình huống có điều kiện, không giả định lịch sử gặp hay ý người kia. Claude review trước khi wiring.</t>
+        </is>
+      </c>
+    </row>
+    <row r="84" ht="26.399999618530273" customHeight="1">
       <c r="A84" s="9" t="inlineStr">
         <is>
           <t>R03-moon-opposition-sun-partner-deep_dive</t>
@@ -58345,11 +58345,11 @@
       </c>
       <c r="F84" s="9" t="inlineStr">
         <is>
-          <t>Một mẫu dễ thấy là những mùa người yêu bận rộn bên ngoài, buổi tối của bạn ở nhà dài ra; đề xuất một tối cố định trong tuần, rồi xem một tháng sau có giữ được không.</t>
-        </is>
-      </c>
-      <c r="G84" s="9" t="n">
-        <v>38</v>
+          <t xml:space="preserve">Nếu người yêu bận bên ngoài lúc bạn mong có buổi tối chung, nói rõ điều mình cần rồi cùng chọn thời gian, vì lịch bận và mong muốn gần nhau cần được hỏi riêng từng người.</t>
+        </is>
+      </c>
+      <c r="G84" s="9">
+        <v>37</v>
       </c>
       <c r="H84" s="9" t="inlineStr">
         <is>
@@ -58358,7 +58358,7 @@
       </c>
       <c r="I84" s="9" t="inlineStr">
         <is>
-          <t>Uỷ quyền 26/10: duyệt bản nháp (giọng deep_dive cho phép tối đa 40 âm tiết). Codex chuốt trước khi wiring</t>
+          <t xml:space="preserve">Uỷ quyền 26/10: duyệt bản nháp; Codex chuốt 26/10 để giữ tình huống có điều kiện, không giả định lịch sử gặp hay ý người kia. Claude review trước khi wiring.</t>
         </is>
       </c>
     </row>
@@ -58452,7 +58452,7 @@
         </is>
       </c>
     </row>
-    <row r="87">
+    <row r="87" ht="26.399999618530273" customHeight="1">
       <c r="A87" s="9" t="inlineStr">
         <is>
           <t>R03-moon-sextile-mercury-friend-deep_dive</t>
@@ -58480,11 +58480,11 @@
       </c>
       <c r="F87" s="9" t="inlineStr">
         <is>
-          <t>Hay gặp ở hai bạn là một tin than thở ngắn của bạn được bạn ấy đáp bằng lời khá trúng; nhắn trước cũng được, miễn là nhìn xem bạn ấy có đang bận hay không.</t>
-        </is>
-      </c>
-      <c r="G87" s="9" t="n">
-        <v>36</v>
+          <t xml:space="preserve">Nếu một tin than thở của bạn được bạn ấy đáp đúng điều đang cần, ghi nhận câu ấy rồi hỏi lúc nào tiện kể tiếp, vì sự lắng nghe cũng cần thời gian của cả hai.</t>
+        </is>
+      </c>
+      <c r="G87" s="9">
+        <v>37</v>
       </c>
       <c r="H87" s="9" t="inlineStr">
         <is>
@@ -58493,7 +58493,7 @@
       </c>
       <c r="I87" s="9" t="inlineStr">
         <is>
-          <t>Uỷ quyền 26/10: duyệt bản nháp (giọng deep_dive cho phép tối đa 40 âm tiết). Codex chuốt trước khi wiring</t>
+          <t xml:space="preserve">Uỷ quyền 26/10: duyệt bản nháp; Codex chuốt 26/10 để giữ tình huống có điều kiện, không giả định lịch sử gặp hay ý người kia. Claude review trước khi wiring.</t>
         </is>
       </c>
     </row>
@@ -58947,7 +58947,7 @@
         </is>
       </c>
     </row>
-    <row r="98">
+    <row r="98" ht="26.399999618530273" customHeight="1">
       <c r="A98" s="9" t="inlineStr">
         <is>
           <t>R03-sun-conjunction-venus-crush-deep_dive</t>
@@ -58975,10 +58975,10 @@
       </c>
       <c r="F98" s="9" t="inlineStr">
         <is>
-          <t>Điều hiện ra là những hôm bạn để lộ nét riêng của mình, crush thường đáp bằng câu hỏi và lời hẹn gặp lại; ghi lại qua vài tuần, vì vài lần trùng hợp chưa thành nếp.</t>
-        </is>
-      </c>
-      <c r="G98" s="9" t="n">
+          <t xml:space="preserve">Khi bạn kể chuyện bằng giọng tự nhiên, để ý cách crush tiếp lời qua nhiều lần và hỏi nếu chưa rõ, vì một câu hỏi thêm chưa có nghĩa là người ấy muốn tiến xa hơn.</t>
+        </is>
+      </c>
+      <c r="G98" s="9">
         <v>37</v>
       </c>
       <c r="H98" s="9" t="inlineStr">
@@ -58988,11 +58988,11 @@
       </c>
       <c r="I98" s="9" t="inlineStr">
         <is>
-          <t>Uỷ quyền 26/10: duyệt bản nháp (giọng deep_dive cho phép tối đa 40 âm tiết). Codex chuốt trước khi wiring; cần chuốt: câu dễ cấn hơi nghiêng về mô tả người kia hoặc ngầm hứa tiến triển</t>
-        </is>
-      </c>
-    </row>
-    <row r="99">
+          <t xml:space="preserve">Uỷ quyền 26/10: duyệt bản nháp; Codex chuốt 26/10 để giữ tình huống có điều kiện, không giả định lịch sử gặp hay ý người kia. Claude review trước khi wiring.</t>
+        </is>
+      </c>
+    </row>
+    <row r="99" ht="26.399999618530273" customHeight="1">
       <c r="A99" s="9" t="inlineStr">
         <is>
           <t>R03-sun-conjunction-venus-friend-deep_dive</t>
@@ -59020,10 +59020,10 @@
       </c>
       <c r="F99" s="9" t="inlineStr">
         <is>
-          <t>Nhìn qua những lần gặp, bạn ấy hay nhớ những chi tiết nhỏ bạn từng kể và nhắc lại đúng lúc; ghi nhận điều đó, rồi xem bạn có làm điều tương tự cho bạn ấy không.</t>
-        </is>
-      </c>
-      <c r="G99" s="9" t="n">
+          <t xml:space="preserve">Nếu bạn ấy nhớ và nhắc lại chi tiết nhỏ bạn từng kể, ghi nhận việc ấy rồi xem mình có lắng nghe tương tự không, vì một tình bạn cần chỗ kể cho cả hai người.</t>
+        </is>
+      </c>
+      <c r="G99" s="9">
         <v>37</v>
       </c>
       <c r="H99" s="9" t="inlineStr">
@@ -59033,7 +59033,7 @@
       </c>
       <c r="I99" s="9" t="inlineStr">
         <is>
-          <t>Uỷ quyền 26/10: duyệt bản nháp (giọng deep_dive cho phép tối đa 40 âm tiết). Codex chuốt trước khi wiring</t>
+          <t xml:space="preserve">Uỷ quyền 26/10: duyệt bản nháp; Codex chuốt 26/10 để giữ tình huống có điều kiện, không giả định lịch sử gặp hay ý người kia. Claude review trước khi wiring.</t>
         </is>
       </c>
     </row>
@@ -59127,7 +59127,7 @@
         </is>
       </c>
     </row>
-    <row r="102">
+    <row r="102" ht="26.399999618530273" customHeight="1">
       <c r="A102" s="9" t="inlineStr">
         <is>
           <t>R03-sun-square-mercury-crush-deep_dive</t>
@@ -59155,10 +59155,10 @@
       </c>
       <c r="F102" s="9" t="inlineStr">
         <is>
-          <t>Chỗ dễ cấn là ngay sau khi bạn khoe một thành quả, crush hay hỏi lại từng chi tiết nhỏ; trả lời trước rồi mới quyết có buồn không, và nhìn cả cuộc chat thay vì một câu.</t>
-        </is>
-      </c>
-      <c r="G102" s="9" t="n">
+          <t xml:space="preserve">Nếu crush hỏi kỹ ngay sau khi bạn khoe thành quả, bạn có thể thấy hụt; nói rõ hôm nay mình muốn chia vui hay xin ý kiến, rồi xem họ đáp, thay vì đoán từ một câu.</t>
+        </is>
+      </c>
+      <c r="G102" s="9">
         <v>38</v>
       </c>
       <c r="H102" s="9" t="inlineStr">
@@ -59168,7 +59168,7 @@
       </c>
       <c r="I102" s="9" t="inlineStr">
         <is>
-          <t>Uỷ quyền 26/10: duyệt bản nháp (giọng deep_dive cho phép tối đa 40 âm tiết). Codex chuốt trước khi wiring</t>
+          <t xml:space="preserve">Uỷ quyền 26/10: duyệt bản nháp; Codex chuốt 26/10 để giữ tình huống có điều kiện, không giả định lịch sử gặp hay ý người kia. Claude review trước khi wiring.</t>
         </is>
       </c>
     </row>
@@ -59307,7 +59307,7 @@
         </is>
       </c>
     </row>
-    <row r="106">
+    <row r="106" ht="26.399999618530273" customHeight="1">
       <c r="A106" s="9" t="inlineStr">
         <is>
           <t>R03-sun-trine-moon-crush-deep_dive</t>
@@ -59335,11 +59335,11 @@
       </c>
       <c r="F106" s="9" t="inlineStr">
         <is>
-          <t>Một quan sát nhẹ là crush thường kể chuyện chậm rãi và dài hơn khi bạn giữ giọng bình thản; xem họ có tự tìm đến bạn để kể không, vì đó mới là tín hiệu rõ.</t>
-        </is>
-      </c>
-      <c r="G106" s="9" t="n">
-        <v>37</v>
+          <t xml:space="preserve">Nếu crush kể dài hơn lúc bạn nói chuyện bình thản, cứ lắng nghe và hỏi họ có muốn kể tiếp, vì một cuộc trò chuyện dễ chịu chưa xác định tình cảm của người kia.</t>
+        </is>
+      </c>
+      <c r="G106" s="9">
+        <v>36</v>
       </c>
       <c r="H106" s="9" t="inlineStr">
         <is>
@@ -59348,11 +59348,11 @@
       </c>
       <c r="I106" s="9" t="inlineStr">
         <is>
-          <t>Uỷ quyền 26/10: duyệt bản nháp (giọng deep_dive cho phép tối đa 40 âm tiết). Codex chuốt trước khi wiring</t>
-        </is>
-      </c>
-    </row>
-    <row r="107">
+          <t xml:space="preserve">Uỷ quyền 26/10: duyệt bản nháp; Codex chuốt 26/10 để giữ tình huống có điều kiện, không giả định lịch sử gặp hay ý người kia. Claude review trước khi wiring.</t>
+        </is>
+      </c>
+    </row>
+    <row r="107" ht="26.399999618530273" customHeight="1">
       <c r="A107" s="9" t="inlineStr">
         <is>
           <t>R03-sun-trine-moon-friend-deep_dive</t>
@@ -59380,11 +59380,11 @@
       </c>
       <c r="F107" s="9" t="inlineStr">
         <is>
-          <t>Nhìn lại những lần gần đây, bạn thường là chỗ bạn ấy ghé qua sau một ngày rối, và buổi gặp hay kết thúc nhẹ nhõm; vai này quý, nhưng cũng cần có ngày bạn được nghe lại.</t>
-        </is>
-      </c>
-      <c r="G107" s="9" t="n">
-        <v>38</v>
+          <t xml:space="preserve">Nếu bạn ấy hay tìm tới bạn sau ngày khó, hỏi lúc này muốn được nghe hay góp ý, và nói rõ khi bạn cần nghỉ, vì quan tâm không đồng nghĩa với luôn có mặt.</t>
+        </is>
+      </c>
+      <c r="G107" s="9">
+        <v>36</v>
       </c>
       <c r="H107" s="9" t="inlineStr">
         <is>
@@ -59393,7 +59393,7 @@
       </c>
       <c r="I107" s="9" t="inlineStr">
         <is>
-          <t>Uỷ quyền 26/10: duyệt bản nháp (giọng deep_dive cho phép tối đa 40 âm tiết). Codex chuốt trước khi wiring</t>
+          <t xml:space="preserve">Uỷ quyền 26/10: duyệt bản nháp; Codex chuốt 26/10 để giữ tình huống có điều kiện, không giả định lịch sử gặp hay ý người kia. Claude review trước khi wiring.</t>
         </is>
       </c>
     </row>
@@ -59487,7 +59487,7 @@
         </is>
       </c>
     </row>
-    <row r="110">
+    <row r="110" ht="26.399999618530273" customHeight="1">
       <c r="A110" s="9" t="inlineStr">
         <is>
           <t>R03-sun-trine-sun-crush-deep_dive</t>
@@ -59515,11 +59515,11 @@
       </c>
       <c r="F110" s="9" t="inlineStr">
         <is>
-          <t>Xét theo những buổi đi chơi, năng lượng của bạn và crush thường lên xuống khá cùng nhịp; thử vài kiểu hoạt động khác nhau, và đừng coi một buổi vui là câu trả lời.</t>
-        </is>
-      </c>
-      <c r="G110" s="9" t="n">
-        <v>35</v>
+          <t xml:space="preserve">Nếu bạn và crush hào hứng với cùng hoạt động, thử một dịp phù hợp cả hai rồi hỏi buổi đó thế nào, vì một lần vui chưa trả lời được toàn bộ chuyện giữa hai người.</t>
+        </is>
+      </c>
+      <c r="G110" s="9">
+        <v>37</v>
       </c>
       <c r="H110" s="9" t="inlineStr">
         <is>
@@ -59528,7 +59528,7 @@
       </c>
       <c r="I110" s="9" t="inlineStr">
         <is>
-          <t>Uỷ quyền 26/10: duyệt bản nháp (giọng deep_dive cho phép tối đa 40 âm tiết). Codex chuốt trước khi wiring</t>
+          <t xml:space="preserve">Uỷ quyền 26/10: duyệt bản nháp; Codex chuốt 26/10 để giữ tình huống có điều kiện, không giả định lịch sử gặp hay ý người kia. Claude review trước khi wiring.</t>
         </is>
       </c>
     </row>
@@ -60567,7 +60567,7 @@
         </is>
       </c>
     </row>
-    <row r="134">
+    <row r="134" ht="26.399999618530273" customHeight="1">
       <c r="A134" s="9" t="inlineStr">
         <is>
           <t>R03-sun-conjunction-true_node-crush-deep_dive</t>
@@ -60595,11 +60595,11 @@
       </c>
       <c r="F134" s="9" t="inlineStr">
         <is>
-          <t>Một điều lớp này ghi lại là vài nếp sống của bạn đôi khi được crush thử theo; vui với điều đó, và nhớ họ đi hướng nào vẫn là lựa chọn của họ.</t>
-        </is>
-      </c>
-      <c r="G134" s="9" t="n">
-        <v>34</v>
+          <t xml:space="preserve">Nếu crush hỏi rồi thử một nếp sống bạn chia sẻ, cứ nói phần hữu ích và để họ làm theo cách riêng, vì việc thử ấy chưa nói lên tình cảm hay hướng họ sẽ chọn.</t>
+        </is>
+      </c>
+      <c r="G134" s="9">
+        <v>37</v>
       </c>
       <c r="H134" s="9" t="inlineStr">
         <is>
@@ -60608,11 +60608,11 @@
       </c>
       <c r="I134" s="9" t="inlineStr">
         <is>
-          <t>Uỷ quyền 26/10: duyệt bản nháp (giọng deep_dive cho phép tối đa 40 âm tiết). Codex chuốt trước khi wiring</t>
-        </is>
-      </c>
-    </row>
-    <row r="135">
+          <t xml:space="preserve">Uỷ quyền 26/10: duyệt bản nháp; Codex chuốt 26/10 để giữ tình huống có điều kiện, không giả định lịch sử gặp hay ý người kia. Claude review trước khi wiring.</t>
+        </is>
+      </c>
+    </row>
+    <row r="135" ht="26.399999618530273" customHeight="1">
       <c r="A135" s="9" t="inlineStr">
         <is>
           <t>R03-sun-conjunction-true_node-friend-deep_dive</t>
@@ -60640,11 +60640,11 @@
       </c>
       <c r="F135" s="9" t="inlineStr">
         <is>
-          <t>Theo những lần gặp, bạn ấy hay mượn vài cách làm của bạn rồi biến tấu theo kiểu riêng; khen phần biến tấu đó, và để bạn ấy tự quyết đi tiếp tới đâu.</t>
-        </is>
-      </c>
-      <c r="G135" s="9" t="n">
-        <v>34</v>
+          <t xml:space="preserve">Nếu bạn ấy thử cách làm của bạn rồi biến tấu, hỏi phần nào phù hợp và ghi nhận lựa chọn riêng ấy, vì chia sẻ kinh nghiệm không có nghĩa là quyết giúp họ bước tiếp theo.</t>
+        </is>
+      </c>
+      <c r="G135" s="9">
+        <v>38</v>
       </c>
       <c r="H135" s="9" t="inlineStr">
         <is>
@@ -60653,7 +60653,7 @@
       </c>
       <c r="I135" s="9" t="inlineStr">
         <is>
-          <t>Uỷ quyền 26/10: duyệt bản nháp (giọng deep_dive cho phép tối đa 40 âm tiết). Codex chuốt trước khi wiring</t>
+          <t xml:space="preserve">Uỷ quyền 26/10: duyệt bản nháp; Codex chuốt 26/10 để giữ tình huống có điều kiện, không giả định lịch sử gặp hay ý người kia. Claude review trước khi wiring.</t>
         </is>
       </c>
     </row>

</xml_diff>